<commit_message>
Replace Editable column with 3-state Mode (Locked/Default/Per-piece)
- Mode dropdown with color-coded rows: gray=Locked, soft yellow=Default,
  soft blue=Per-piece
- New Legend tab explains each mode and where the value lives
- Counts: 6 Locked, 66 Default, 11 Per-piece across all 83 fields

The Default mode captures fields that are technically editable but
behave as static defaults — populated once on the Verticals table and
only overridden per-piece when needed.

https://claude.ai/code/session_01TDpKdzUTk2mGVaLmXs7jGf
</commit_message>
<xml_diff>
--- a/markup/field_specs.xlsx
+++ b/markup/field_specs.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="Field Specs" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Open Questions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Legend" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Open Questions" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Field Specs'!$A$1:$N$84</definedName>
@@ -38,7 +39,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -48,6 +49,21 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F3D2B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ECEFF1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF8E1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E1F5FE"/>
       </patternFill>
     </fill>
   </fills>
@@ -63,7 +79,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -72,11 +88,41 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="5">
+  <dxfs count="7">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00ECEFF1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFF8E1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00E1F5FE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -102,13 +148,6 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00BBDEFB"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00ECEFF1"/>
         </patternFill>
       </fill>
     </dxf>
@@ -482,7 +521,7 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="36" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="50" customWidth="1" min="9" max="9"/>
@@ -521,7 +560,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Editable</t>
+          <t>Mode</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -565,7 +604,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="42" customHeight="1">
+    <row r="2" ht="44" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>1</t>
@@ -593,7 +632,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Locked</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -626,10 +665,8 @@
           <t>Locked — brand asset baked into template</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-    </row>
-    <row r="3" ht="42" customHeight="1">
+    </row>
+    <row r="3" ht="44" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>2</t>
@@ -657,7 +694,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -690,10 +727,8 @@
           <t>Drives both #2 and #30 (page 2 section header)</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-    </row>
-    <row r="4" ht="42" customHeight="1">
+    </row>
+    <row r="4" ht="44" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>3</t>
@@ -721,7 +756,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -754,10 +789,8 @@
           <t>Three-beat rhythm matches brand voice</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-    </row>
-    <row r="5" ht="42" customHeight="1">
+    </row>
+    <row r="5" ht="44" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>4</t>
@@ -785,7 +818,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -818,10 +851,8 @@
           <t>Right-half of the dark green header band</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-    </row>
-    <row r="6" ht="42" customHeight="1">
+    </row>
+    <row r="6" ht="44" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>5</t>
@@ -849,7 +880,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -882,10 +913,8 @@
           <t>Plain text — no bold needed</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-    </row>
-    <row r="7" ht="42" customHeight="1">
+    </row>
+    <row r="7" ht="44" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>6</t>
@@ -913,7 +942,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -946,10 +975,8 @@
           <t>Markdown bold supported</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-    </row>
-    <row r="8" ht="42" customHeight="1">
+    </row>
+    <row r="8" ht="44" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>7</t>
@@ -977,7 +1004,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Locked</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1010,10 +1037,8 @@
           <t>Locked — same on every piece</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-    </row>
-    <row r="9" ht="42" customHeight="1">
+    </row>
+    <row r="9" ht="44" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>8</t>
@@ -1041,7 +1066,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -1070,10 +1095,8 @@
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-    </row>
-    <row r="10" ht="42" customHeight="1">
+    </row>
+    <row r="10" ht="44" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>9</t>
@@ -1101,7 +1124,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1130,10 +1153,8 @@
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-    </row>
-    <row r="11" ht="42" customHeight="1">
+    </row>
+    <row r="11" ht="44" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
           <t>10</t>
@@ -1161,7 +1182,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -1190,10 +1211,8 @@
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-    </row>
-    <row r="12" ht="42" customHeight="1">
+    </row>
+    <row r="12" ht="44" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
           <t>11</t>
@@ -1221,7 +1240,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1250,10 +1269,8 @@
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-    </row>
-    <row r="13" ht="42" customHeight="1">
+    </row>
+    <row r="13" ht="44" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
           <t>12</t>
@@ -1281,7 +1298,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -1310,10 +1327,8 @@
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-    </row>
-    <row r="14" ht="42" customHeight="1">
+    </row>
+    <row r="14" ht="44" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
           <t>13</t>
@@ -1341,7 +1356,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1370,10 +1385,8 @@
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-    </row>
-    <row r="15" ht="42" customHeight="1">
+    </row>
+    <row r="15" ht="44" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
           <t>14</t>
@@ -1401,7 +1414,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -1430,10 +1443,8 @@
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
-    </row>
-    <row r="16" ht="42" customHeight="1">
+    </row>
+    <row r="16" ht="44" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
           <t>15</t>
@@ -1461,7 +1472,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -1490,10 +1501,8 @@
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
-    </row>
-    <row r="17" ht="42" customHeight="1">
+    </row>
+    <row r="17" ht="44" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
           <t>16</t>
@@ -1521,7 +1530,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Locked</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -1554,10 +1563,8 @@
           <t>Locked — green panel header</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
-    </row>
-    <row r="18" ht="42" customHeight="1">
+    </row>
+    <row r="18" ht="44" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
           <t>17</t>
@@ -1585,7 +1592,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -1614,10 +1621,8 @@
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
-    </row>
-    <row r="19" ht="42" customHeight="1">
+    </row>
+    <row r="19" ht="44" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
           <t>18</t>
@@ -1645,7 +1650,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -1674,10 +1679,8 @@
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
-    </row>
-    <row r="20" ht="42" customHeight="1">
+    </row>
+    <row r="20" ht="44" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
           <t>19</t>
@@ -1705,7 +1708,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -1734,10 +1737,8 @@
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-    </row>
-    <row r="21" ht="42" customHeight="1">
+    </row>
+    <row r="21" ht="44" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
           <t>20</t>
@@ -1765,7 +1766,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -1794,10 +1795,8 @@
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr"/>
-    </row>
-    <row r="22" ht="42" customHeight="1">
+    </row>
+    <row r="22" ht="44" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
           <t>21</t>
@@ -1825,7 +1824,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Per-piece</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -1858,10 +1857,8 @@
           <t>Distinct from stats 1–4 because it's recipient-specific</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
-    </row>
-    <row r="23" ht="42" customHeight="1">
+    </row>
+    <row r="23" ht="44" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
           <t>22</t>
@@ -1889,7 +1886,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Per-piece</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -1922,10 +1919,8 @@
           <t>Bottom of green panel</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
-    </row>
-    <row r="24" ht="42" customHeight="1">
+    </row>
+    <row r="24" ht="44" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
           <t>23</t>
@@ -1953,7 +1948,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Per-piece</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -1986,10 +1981,8 @@
           <t>Same on all 3 pages</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
-    </row>
-    <row r="25" ht="42" customHeight="1">
+    </row>
+    <row r="25" ht="44" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
           <t>24</t>
@@ -2017,7 +2010,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Per-piece</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -2046,10 +2039,8 @@
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-    </row>
-    <row r="26" ht="42" customHeight="1">
+    </row>
+    <row r="26" ht="44" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
           <t>25</t>
@@ -2077,7 +2068,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Per-piece</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -2106,10 +2097,8 @@
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
-    </row>
-    <row r="27" ht="42" customHeight="1">
+    </row>
+    <row r="27" ht="44" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
           <t>26</t>
@@ -2137,7 +2126,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Per-piece</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -2166,10 +2155,8 @@
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
-    </row>
-    <row r="28" ht="42" customHeight="1">
+    </row>
+    <row r="28" ht="44" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
           <t>27</t>
@@ -2197,7 +2184,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Per-piece</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -2230,10 +2217,8 @@
           <t>Auto-generated from URL → image</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
-    </row>
-    <row r="29" ht="42" customHeight="1">
+    </row>
+    <row r="29" ht="44" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
           <t>28</t>
@@ -2261,7 +2246,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -2294,10 +2279,8 @@
           <t>Full-width banner</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
-    </row>
-    <row r="30" ht="42" customHeight="1">
+    </row>
+    <row r="30" ht="44" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
           <t>29</t>
@@ -2325,7 +2308,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -2354,10 +2337,8 @@
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr"/>
-      <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr"/>
-    </row>
-    <row r="31" ht="42" customHeight="1">
+    </row>
+    <row r="31" ht="44" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
           <t>30</t>
@@ -2385,7 +2366,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Locked</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -2418,10 +2399,8 @@
           <t>Locked template; vertical name mirrors #2</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
-    </row>
-    <row r="32" ht="42" customHeight="1">
+    </row>
+    <row r="32" ht="44" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
           <t>31</t>
@@ -2449,7 +2428,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -2478,10 +2457,8 @@
         </is>
       </c>
       <c r="L32" s="2" t="inlineStr"/>
-      <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr"/>
-    </row>
-    <row r="33" ht="42" customHeight="1">
+    </row>
+    <row r="33" ht="44" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
           <t>32</t>
@@ -2509,7 +2486,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -2538,10 +2515,8 @@
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr"/>
-      <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr"/>
-    </row>
-    <row r="34" ht="42" customHeight="1">
+    </row>
+    <row r="34" ht="44" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
           <t>33</t>
@@ -2569,7 +2544,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -2598,10 +2573,8 @@
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr"/>
-      <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr"/>
-    </row>
-    <row r="35" ht="42" customHeight="1">
+    </row>
+    <row r="35" ht="44" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
           <t>34</t>
@@ -2629,7 +2602,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -2658,10 +2631,8 @@
         </is>
       </c>
       <c r="L35" s="2" t="inlineStr"/>
-      <c r="M35" t="inlineStr"/>
-      <c r="N35" t="inlineStr"/>
-    </row>
-    <row r="36" ht="42" customHeight="1">
+    </row>
+    <row r="36" ht="44" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
           <t>35</t>
@@ -2689,7 +2660,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -2718,10 +2689,8 @@
         </is>
       </c>
       <c r="L36" s="2" t="inlineStr"/>
-      <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
-    </row>
-    <row r="37" ht="42" customHeight="1">
+    </row>
+    <row r="37" ht="44" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
           <t>36</t>
@@ -2749,7 +2718,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -2778,10 +2747,8 @@
         </is>
       </c>
       <c r="L37" s="2" t="inlineStr"/>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr"/>
-    </row>
-    <row r="38" ht="42" customHeight="1">
+    </row>
+    <row r="38" ht="44" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
           <t>37</t>
@@ -2809,7 +2776,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -2838,10 +2805,8 @@
         </is>
       </c>
       <c r="L38" s="2" t="inlineStr"/>
-      <c r="M38" t="inlineStr"/>
-      <c r="N38" t="inlineStr"/>
-    </row>
-    <row r="39" ht="42" customHeight="1">
+    </row>
+    <row r="39" ht="44" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
           <t>38</t>
@@ -2869,7 +2834,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -2898,10 +2863,8 @@
         </is>
       </c>
       <c r="L39" s="2" t="inlineStr"/>
-      <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr"/>
-    </row>
-    <row r="40" ht="42" customHeight="1">
+    </row>
+    <row r="40" ht="44" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
           <t>39</t>
@@ -2929,7 +2892,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -2958,10 +2921,8 @@
         </is>
       </c>
       <c r="L40" s="2" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr"/>
-    </row>
-    <row r="41" ht="42" customHeight="1">
+    </row>
+    <row r="41" ht="44" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
         <is>
           <t>40</t>
@@ -2989,7 +2950,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -3018,10 +2979,8 @@
         </is>
       </c>
       <c r="L41" s="2" t="inlineStr"/>
-      <c r="M41" t="inlineStr"/>
-      <c r="N41" t="inlineStr"/>
-    </row>
-    <row r="42" ht="42" customHeight="1">
+    </row>
+    <row r="42" ht="44" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
           <t>41</t>
@@ -3049,7 +3008,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -3078,10 +3037,8 @@
         </is>
       </c>
       <c r="L42" s="2" t="inlineStr"/>
-      <c r="M42" t="inlineStr"/>
-      <c r="N42" t="inlineStr"/>
-    </row>
-    <row r="43" ht="42" customHeight="1">
+    </row>
+    <row r="43" ht="44" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
         <is>
           <t>42</t>
@@ -3109,7 +3066,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -3138,10 +3095,8 @@
         </is>
       </c>
       <c r="L43" s="2" t="inlineStr"/>
-      <c r="M43" t="inlineStr"/>
-      <c r="N43" t="inlineStr"/>
-    </row>
-    <row r="44" ht="42" customHeight="1">
+    </row>
+    <row r="44" ht="44" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
         <is>
           <t>43</t>
@@ -3169,7 +3124,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -3198,10 +3153,8 @@
         </is>
       </c>
       <c r="L44" s="2" t="inlineStr"/>
-      <c r="M44" t="inlineStr"/>
-      <c r="N44" t="inlineStr"/>
-    </row>
-    <row r="45" ht="42" customHeight="1">
+    </row>
+    <row r="45" ht="44" customHeight="1">
       <c r="A45" s="2" t="inlineStr">
         <is>
           <t>44</t>
@@ -3229,7 +3182,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -3258,10 +3211,8 @@
         </is>
       </c>
       <c r="L45" s="2" t="inlineStr"/>
-      <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr"/>
-    </row>
-    <row r="46" ht="42" customHeight="1">
+    </row>
+    <row r="46" ht="44" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
         <is>
           <t>45</t>
@@ -3289,7 +3240,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -3318,10 +3269,8 @@
         </is>
       </c>
       <c r="L46" s="2" t="inlineStr"/>
-      <c r="M46" t="inlineStr"/>
-      <c r="N46" t="inlineStr"/>
-    </row>
-    <row r="47" ht="42" customHeight="1">
+    </row>
+    <row r="47" ht="44" customHeight="1">
       <c r="A47" s="2" t="inlineStr">
         <is>
           <t>46</t>
@@ -3349,7 +3298,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -3378,10 +3327,8 @@
         </is>
       </c>
       <c r="L47" s="2" t="inlineStr"/>
-      <c r="M47" t="inlineStr"/>
-      <c r="N47" t="inlineStr"/>
-    </row>
-    <row r="48" ht="42" customHeight="1">
+    </row>
+    <row r="48" ht="44" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
         <is>
           <t>47</t>
@@ -3409,7 +3356,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -3438,10 +3385,8 @@
         </is>
       </c>
       <c r="L48" s="2" t="inlineStr"/>
-      <c r="M48" t="inlineStr"/>
-      <c r="N48" t="inlineStr"/>
-    </row>
-    <row r="49" ht="42" customHeight="1">
+    </row>
+    <row r="49" ht="44" customHeight="1">
       <c r="A49" s="2" t="inlineStr">
         <is>
           <t>48</t>
@@ -3469,7 +3414,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -3498,10 +3443,8 @@
         </is>
       </c>
       <c r="L49" s="2" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
-      <c r="N49" t="inlineStr"/>
-    </row>
-    <row r="50" ht="42" customHeight="1">
+    </row>
+    <row r="50" ht="44" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
         <is>
           <t>49</t>
@@ -3529,7 +3472,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -3558,10 +3501,8 @@
         </is>
       </c>
       <c r="L50" s="2" t="inlineStr"/>
-      <c r="M50" t="inlineStr"/>
-      <c r="N50" t="inlineStr"/>
-    </row>
-    <row r="51" ht="42" customHeight="1">
+    </row>
+    <row r="51" ht="44" customHeight="1">
       <c r="A51" s="2" t="inlineStr">
         <is>
           <t>50</t>
@@ -3589,7 +3530,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -3618,10 +3559,8 @@
         </is>
       </c>
       <c r="L51" s="2" t="inlineStr"/>
-      <c r="M51" t="inlineStr"/>
-      <c r="N51" t="inlineStr"/>
-    </row>
-    <row r="52" ht="42" customHeight="1">
+    </row>
+    <row r="52" ht="44" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
         <is>
           <t>51</t>
@@ -3649,7 +3588,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -3678,10 +3617,8 @@
         </is>
       </c>
       <c r="L52" s="2" t="inlineStr"/>
-      <c r="M52" t="inlineStr"/>
-      <c r="N52" t="inlineStr"/>
-    </row>
-    <row r="53" ht="42" customHeight="1">
+    </row>
+    <row r="53" ht="44" customHeight="1">
       <c r="A53" s="2" t="inlineStr">
         <is>
           <t>52</t>
@@ -3709,7 +3646,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -3738,10 +3675,8 @@
         </is>
       </c>
       <c r="L53" s="2" t="inlineStr"/>
-      <c r="M53" t="inlineStr"/>
-      <c r="N53" t="inlineStr"/>
-    </row>
-    <row r="54" ht="42" customHeight="1">
+    </row>
+    <row r="54" ht="44" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
         <is>
           <t>53</t>
@@ -3769,7 +3704,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -3798,10 +3733,8 @@
         </is>
       </c>
       <c r="L54" s="2" t="inlineStr"/>
-      <c r="M54" t="inlineStr"/>
-      <c r="N54" t="inlineStr"/>
-    </row>
-    <row r="55" ht="42" customHeight="1">
+    </row>
+    <row r="55" ht="44" customHeight="1">
       <c r="A55" s="2" t="inlineStr">
         <is>
           <t>54</t>
@@ -3829,7 +3762,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -3858,10 +3791,8 @@
         </is>
       </c>
       <c r="L55" s="2" t="inlineStr"/>
-      <c r="M55" t="inlineStr"/>
-      <c r="N55" t="inlineStr"/>
-    </row>
-    <row r="56" ht="42" customHeight="1">
+    </row>
+    <row r="56" ht="44" customHeight="1">
       <c r="A56" s="2" t="inlineStr">
         <is>
           <t>55</t>
@@ -3889,7 +3820,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Locked</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -3922,10 +3853,8 @@
           <t>Locked — compliance/legal language</t>
         </is>
       </c>
-      <c r="M56" t="inlineStr"/>
-      <c r="N56" t="inlineStr"/>
-    </row>
-    <row r="57" ht="42" customHeight="1">
+    </row>
+    <row r="57" ht="44" customHeight="1">
       <c r="A57" s="2" t="inlineStr">
         <is>
           <t>56</t>
@@ -3953,7 +3882,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Per-piece</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -3986,10 +3915,8 @@
           <t>Mirrors page 1 footer</t>
         </is>
       </c>
-      <c r="M57" t="inlineStr"/>
-      <c r="N57" t="inlineStr"/>
-    </row>
-    <row r="58" ht="42" customHeight="1">
+    </row>
+    <row r="58" ht="44" customHeight="1">
       <c r="A58" s="2" t="inlineStr">
         <is>
           <t>57</t>
@@ -4017,7 +3944,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Per-piece</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -4050,10 +3977,8 @@
           <t>Same QR as page 1</t>
         </is>
       </c>
-      <c r="M58" t="inlineStr"/>
-      <c r="N58" t="inlineStr"/>
-    </row>
-    <row r="59" ht="42" customHeight="1">
+    </row>
+    <row r="59" ht="44" customHeight="1">
       <c r="A59" s="2" t="inlineStr">
         <is>
           <t>58</t>
@@ -4081,7 +4006,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -4110,10 +4035,8 @@
         </is>
       </c>
       <c r="L59" s="2" t="inlineStr"/>
-      <c r="M59" t="inlineStr"/>
-      <c r="N59" t="inlineStr"/>
-    </row>
-    <row r="60" ht="42" customHeight="1">
+    </row>
+    <row r="60" ht="44" customHeight="1">
       <c r="A60" s="2" t="inlineStr">
         <is>
           <t>59</t>
@@ -4141,7 +4064,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Locked</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -4174,10 +4097,8 @@
           <t>Locked</t>
         </is>
       </c>
-      <c r="M60" t="inlineStr"/>
-      <c r="N60" t="inlineStr"/>
-    </row>
-    <row r="61" ht="42" customHeight="1">
+    </row>
+    <row r="61" ht="44" customHeight="1">
       <c r="A61" s="2" t="inlineStr">
         <is>
           <t>60</t>
@@ -4205,7 +4126,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -4234,10 +4155,8 @@
         </is>
       </c>
       <c r="L61" s="2" t="inlineStr"/>
-      <c r="M61" t="inlineStr"/>
-      <c r="N61" t="inlineStr"/>
-    </row>
-    <row r="62" ht="42" customHeight="1">
+    </row>
+    <row r="62" ht="44" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
         <is>
           <t>61</t>
@@ -4265,7 +4184,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -4294,10 +4213,8 @@
         </is>
       </c>
       <c r="L62" s="2" t="inlineStr"/>
-      <c r="M62" t="inlineStr"/>
-      <c r="N62" t="inlineStr"/>
-    </row>
-    <row r="63" ht="42" customHeight="1">
+    </row>
+    <row r="63" ht="44" customHeight="1">
       <c r="A63" s="2" t="inlineStr">
         <is>
           <t>62</t>
@@ -4325,7 +4242,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -4354,10 +4271,8 @@
         </is>
       </c>
       <c r="L63" s="2" t="inlineStr"/>
-      <c r="M63" t="inlineStr"/>
-      <c r="N63" t="inlineStr"/>
-    </row>
-    <row r="64" ht="42" customHeight="1">
+    </row>
+    <row r="64" ht="44" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
         <is>
           <t>63</t>
@@ -4385,7 +4300,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -4414,10 +4329,8 @@
         </is>
       </c>
       <c r="L64" s="2" t="inlineStr"/>
-      <c r="M64" t="inlineStr"/>
-      <c r="N64" t="inlineStr"/>
-    </row>
-    <row r="65" ht="42" customHeight="1">
+    </row>
+    <row r="65" ht="44" customHeight="1">
       <c r="A65" s="2" t="inlineStr">
         <is>
           <t>64</t>
@@ -4445,7 +4358,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -4474,10 +4387,8 @@
         </is>
       </c>
       <c r="L65" s="2" t="inlineStr"/>
-      <c r="M65" t="inlineStr"/>
-      <c r="N65" t="inlineStr"/>
-    </row>
-    <row r="66" ht="42" customHeight="1">
+    </row>
+    <row r="66" ht="44" customHeight="1">
       <c r="A66" s="2" t="inlineStr">
         <is>
           <t>65</t>
@@ -4505,7 +4416,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -4534,10 +4445,8 @@
         </is>
       </c>
       <c r="L66" s="2" t="inlineStr"/>
-      <c r="M66" t="inlineStr"/>
-      <c r="N66" t="inlineStr"/>
-    </row>
-    <row r="67" ht="42" customHeight="1">
+    </row>
+    <row r="67" ht="44" customHeight="1">
       <c r="A67" s="2" t="inlineStr">
         <is>
           <t>66</t>
@@ -4565,7 +4474,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -4594,10 +4503,8 @@
         </is>
       </c>
       <c r="L67" s="2" t="inlineStr"/>
-      <c r="M67" t="inlineStr"/>
-      <c r="N67" t="inlineStr"/>
-    </row>
-    <row r="68" ht="42" customHeight="1">
+    </row>
+    <row r="68" ht="44" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
         <is>
           <t>67</t>
@@ -4625,7 +4532,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -4654,10 +4561,8 @@
         </is>
       </c>
       <c r="L68" s="2" t="inlineStr"/>
-      <c r="M68" t="inlineStr"/>
-      <c r="N68" t="inlineStr"/>
-    </row>
-    <row r="69" ht="42" customHeight="1">
+    </row>
+    <row r="69" ht="44" customHeight="1">
       <c r="A69" s="2" t="inlineStr">
         <is>
           <t>68</t>
@@ -4685,7 +4590,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -4714,10 +4619,8 @@
         </is>
       </c>
       <c r="L69" s="2" t="inlineStr"/>
-      <c r="M69" t="inlineStr"/>
-      <c r="N69" t="inlineStr"/>
-    </row>
-    <row r="70" ht="42" customHeight="1">
+    </row>
+    <row r="70" ht="44" customHeight="1">
       <c r="A70" s="2" t="inlineStr">
         <is>
           <t>69</t>
@@ -4745,7 +4648,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -4774,10 +4677,8 @@
         </is>
       </c>
       <c r="L70" s="2" t="inlineStr"/>
-      <c r="M70" t="inlineStr"/>
-      <c r="N70" t="inlineStr"/>
-    </row>
-    <row r="71" ht="42" customHeight="1">
+    </row>
+    <row r="71" ht="44" customHeight="1">
       <c r="A71" s="2" t="inlineStr">
         <is>
           <t>70</t>
@@ -4805,7 +4706,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -4834,10 +4735,8 @@
         </is>
       </c>
       <c r="L71" s="2" t="inlineStr"/>
-      <c r="M71" t="inlineStr"/>
-      <c r="N71" t="inlineStr"/>
-    </row>
-    <row r="72" ht="42" customHeight="1">
+    </row>
+    <row r="72" ht="44" customHeight="1">
       <c r="A72" s="2" t="inlineStr">
         <is>
           <t>71</t>
@@ -4865,7 +4764,7 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -4894,10 +4793,8 @@
         </is>
       </c>
       <c r="L72" s="2" t="inlineStr"/>
-      <c r="M72" t="inlineStr"/>
-      <c r="N72" t="inlineStr"/>
-    </row>
-    <row r="73" ht="42" customHeight="1">
+    </row>
+    <row r="73" ht="44" customHeight="1">
       <c r="A73" s="2" t="inlineStr">
         <is>
           <t>72</t>
@@ -4925,7 +4822,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -4954,10 +4851,8 @@
         </is>
       </c>
       <c r="L73" s="2" t="inlineStr"/>
-      <c r="M73" t="inlineStr"/>
-      <c r="N73" t="inlineStr"/>
-    </row>
-    <row r="74" ht="42" customHeight="1">
+    </row>
+    <row r="74" ht="44" customHeight="1">
       <c r="A74" s="2" t="inlineStr">
         <is>
           <t>73</t>
@@ -4985,7 +4880,7 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -5014,10 +4909,8 @@
         </is>
       </c>
       <c r="L74" s="2" t="inlineStr"/>
-      <c r="M74" t="inlineStr"/>
-      <c r="N74" t="inlineStr"/>
-    </row>
-    <row r="75" ht="42" customHeight="1">
+    </row>
+    <row r="75" ht="44" customHeight="1">
       <c r="A75" s="2" t="inlineStr">
         <is>
           <t>74</t>
@@ -5045,7 +4938,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -5074,10 +4967,8 @@
         </is>
       </c>
       <c r="L75" s="2" t="inlineStr"/>
-      <c r="M75" t="inlineStr"/>
-      <c r="N75" t="inlineStr"/>
-    </row>
-    <row r="76" ht="42" customHeight="1">
+    </row>
+    <row r="76" ht="44" customHeight="1">
       <c r="A76" s="2" t="inlineStr">
         <is>
           <t>75</t>
@@ -5105,7 +4996,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -5134,10 +5025,8 @@
         </is>
       </c>
       <c r="L76" s="2" t="inlineStr"/>
-      <c r="M76" t="inlineStr"/>
-      <c r="N76" t="inlineStr"/>
-    </row>
-    <row r="77" ht="42" customHeight="1">
+    </row>
+    <row r="77" ht="44" customHeight="1">
       <c r="A77" s="2" t="inlineStr">
         <is>
           <t>76</t>
@@ -5165,7 +5054,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -5194,10 +5083,8 @@
         </is>
       </c>
       <c r="L77" s="2" t="inlineStr"/>
-      <c r="M77" t="inlineStr"/>
-      <c r="N77" t="inlineStr"/>
-    </row>
-    <row r="78" ht="42" customHeight="1">
+    </row>
+    <row r="78" ht="44" customHeight="1">
       <c r="A78" s="2" t="inlineStr">
         <is>
           <t>77</t>
@@ -5225,7 +5112,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -5258,10 +5145,8 @@
           <t>Markdown bold supported</t>
         </is>
       </c>
-      <c r="M78" t="inlineStr"/>
-      <c r="N78" t="inlineStr"/>
-    </row>
-    <row r="79" ht="42" customHeight="1">
+    </row>
+    <row r="79" ht="44" customHeight="1">
       <c r="A79" s="2" t="inlineStr">
         <is>
           <t>78</t>
@@ -5289,7 +5174,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -5322,10 +5207,8 @@
           <t>Sits inside dark green CTA block</t>
         </is>
       </c>
-      <c r="M79" t="inlineStr"/>
-      <c r="N79" t="inlineStr"/>
-    </row>
-    <row r="80" ht="42" customHeight="1">
+    </row>
+    <row r="80" ht="44" customHeight="1">
       <c r="A80" s="2" t="inlineStr">
         <is>
           <t>79</t>
@@ -5353,7 +5236,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -5382,10 +5265,8 @@
         </is>
       </c>
       <c r="L80" s="2" t="inlineStr"/>
-      <c r="M80" t="inlineStr"/>
-      <c r="N80" t="inlineStr"/>
-    </row>
-    <row r="81" ht="42" customHeight="1">
+    </row>
+    <row r="81" ht="44" customHeight="1">
       <c r="A81" s="2" t="inlineStr">
         <is>
           <t>80</t>
@@ -5413,7 +5294,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -5442,10 +5323,8 @@
         </is>
       </c>
       <c r="L81" s="2" t="inlineStr"/>
-      <c r="M81" t="inlineStr"/>
-      <c r="N81" t="inlineStr"/>
-    </row>
-    <row r="82" ht="42" customHeight="1">
+    </row>
+    <row r="82" ht="44" customHeight="1">
       <c r="A82" s="2" t="inlineStr">
         <is>
           <t>81</t>
@@ -5473,7 +5352,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -5502,10 +5381,8 @@
         </is>
       </c>
       <c r="L82" s="2" t="inlineStr"/>
-      <c r="M82" t="inlineStr"/>
-      <c r="N82" t="inlineStr"/>
-    </row>
-    <row r="83" ht="42" customHeight="1">
+    </row>
+    <row r="83" ht="44" customHeight="1">
       <c r="A83" s="2" t="inlineStr">
         <is>
           <t>82</t>
@@ -5533,7 +5410,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Per-piece</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -5566,10 +5443,8 @@
           <t>Mirrors page 1 footer</t>
         </is>
       </c>
-      <c r="M83" t="inlineStr"/>
-      <c r="N83" t="inlineStr"/>
-    </row>
-    <row r="84" ht="42" customHeight="1">
+    </row>
+    <row r="84" ht="44" customHeight="1">
       <c r="A84" s="2" t="inlineStr">
         <is>
           <t>83</t>
@@ -5597,7 +5472,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Per-piece</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -5630,36 +5505,48 @@
           <t>Same QR as page 1</t>
         </is>
       </c>
-      <c r="M84" t="inlineStr"/>
-      <c r="N84" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:N84"/>
+  <conditionalFormatting sqref="F2:F84">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Locked"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"Default"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
+      <formula>"Per-piece"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2:N84">
+    <cfRule type="expression" priority="4" dxfId="0">
+      <formula>$F2="Locked"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" dxfId="2">
+      <formula>$F2="Per-piece"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="M2:M84">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="3">
       <formula>"Approved"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="7" operator="equal" dxfId="4">
       <formula>"Needs Edit"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
+    <cfRule type="cellIs" priority="8" operator="equal" dxfId="5">
       <formula>"Remove"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
+    <cfRule type="cellIs" priority="9" operator="equal" dxfId="6">
       <formula>"Open Question"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:N84">
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
-      <formula>$F2="No"</formula>
-    </cfRule>
-  </conditionalFormatting>
   <dataValidations count="2">
+    <dataValidation sqref="F2:F84" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Locked,Default,Per-piece"</formula1>
+    </dataValidation>
     <dataValidation sqref="M2:M84" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Approved,Needs Edit,Remove,Open Question"</formula1>
-    </dataValidation>
-    <dataValidation sqref="F2:F84" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5667,6 +5554,114 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Mode</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Meaning</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Where value lives</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Behavior</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="56" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Cannot be changed without editing the template code</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Hardcoded in template.html</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Same on every piece</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="56" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Default</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Has a baked-in default; can be overridden per-piece but usually isn't</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Verticals table (default) + optional override on Collateral table</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>If Collateral override is blank → use Vertical default. If filled → use override.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="56" customHeight="1">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Per-piece</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Set on every Collateral record (no default)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Collateral table (or linked Reps record)</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Always varies</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Rename 'Airtable Field' column to 'Field Name'
</commit_message>
<xml_diff>
--- a/markup/field_specs.xlsx
+++ b/markup/field_specs.xlsx
@@ -9,7 +9,6 @@
   <sheets>
     <sheet name="Field Specs" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Legend" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Open Questions" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Field Specs'!$A$1:$N$84</definedName>
@@ -112,14 +111,14 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00FFF8E1"/>
+          <fgColor rgb="00E1F5FE"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00E1F5FE"/>
+          <fgColor rgb="00FFF8E1"/>
         </patternFill>
       </fill>
     </dxf>
@@ -570,7 +569,7 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Airtable Field</t>
+          <t>Field Name</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
@@ -5508,36 +5507,30 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:N84"/>
-  <conditionalFormatting sqref="F2:F84">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
-      <formula>"Locked"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
-      <formula>"Default"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
-      <formula>"Per-piece"</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="A2:N84">
-    <cfRule type="expression" priority="4" dxfId="0">
+    <cfRule type="expression" priority="1" dxfId="0">
       <formula>$F2="Locked"</formula>
     </cfRule>
-    <cfRule type="expression" priority="5" dxfId="2">
+    <cfRule type="expression" priority="2" dxfId="1">
       <formula>$F2="Per-piece"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="F2:F84">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
+      <formula>"Default"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="M2:M84">
-    <cfRule type="cellIs" priority="6" operator="equal" dxfId="3">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
       <formula>"Approved"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="7" operator="equal" dxfId="4">
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
       <formula>"Needs Edit"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="8" operator="equal" dxfId="5">
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="5">
       <formula>"Remove"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="9" operator="equal" dxfId="6">
+    <cfRule type="cellIs" priority="7" operator="equal" dxfId="6">
       <formula>"Open Question"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5625,12 +5618,12 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Verticals table (default) + optional override on Collateral table</t>
+          <t>Inherited from a starter set (or fed in by upstream pipeline)</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>If Collateral override is blank → use Vertical default. If filled → use override.</t>
+          <t>If override is blank → use default. If filled → use override.</t>
         </is>
       </c>
     </row>
@@ -5642,12 +5635,12 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Set on every Collateral record (no default)</t>
+          <t>Set on every PDF (no default)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Collateral table (or linked Reps record)</t>
+          <t>Filled per-account by upstream pipeline</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -5655,160 +5648,6 @@
           <t>Always varies</t>
         </is>
       </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B1" s="3" t="inlineStr">
-        <is>
-          <t>Question</t>
-        </is>
-      </c>
-      <c r="C1" s="3" t="inlineStr">
-        <is>
-          <t>Why it matters</t>
-        </is>
-      </c>
-      <c r="D1" s="3" t="inlineStr">
-        <is>
-          <t>Your answer</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="48" customHeight="1">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Always exactly 8 products on page 2, or variable (4/6/8)?</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Determines if Products is a fixed object or a variable linked list</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr"/>
-    </row>
-    <row r="3" ht="48" customHeight="1">
-      <c r="A3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Always exactly 8 rows in the feature table, or variable?</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Same — fixed vs linked list</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr"/>
-    </row>
-    <row r="4" ht="48" customHeight="1">
-      <c r="A4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Accent color — always dark green or per-vertical?</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Determines if 'Accent color' belongs on Verticals table</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr"/>
-    </row>
-    <row r="5" ht="48" customHeight="1">
-      <c r="A5" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Footer rep info — single Rep record drives all 3 pages?</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Confirms one rep linked record per Collateral row</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr"/>
-    </row>
-    <row r="6" ht="48" customHeight="1">
-      <c r="A6" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>QR target URL — per rep, per collateral piece, or per campaign?</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Determines where the URL field lives (Reps vs Collateral vs both)</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr"/>
-    </row>
-    <row r="7" ht="48" customHeight="1">
-      <c r="A7" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Sensor diagram (#22) — swaps per region/city, or stays national?</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>If per-region, it lives on Collateral, not Verticals</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr"/>
-    </row>
-    <row r="8" ht="48" customHeight="1">
-      <c r="A8" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Page count — always exactly 3, or can verticals drop/add pages?</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Affects template structure (3 fixed pages vs page registry)</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>